<commit_message>
Updated test_DATF with new changes
</commit_message>
<xml_diff>
--- a/DAQEAI_Codebase_Apr2026/datf_core/test/testprotocol/testDATF.xlsx
+++ b/DAQEAI_Codebase_Apr2026/datf_core/test/testprotocol/testDATF.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naveen.natarajan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naveen.natarajan\Downloads\DAQEAI_Codebase_Apr2026\DAQEAI_Codebase_Apr2026\datf_core\test\testprotocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263D536B-9CD5-48A4-A82D-342E6D5B2F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD831D8-B6C9-4A63-961C-E1C66F165C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -273,10 +273,10 @@
     <t>test/data/source</t>
   </si>
   <si>
-    <t>test_DATF</t>
-  </si>
-  <si>
     <t>testcase1</t>
+  </si>
+  <si>
+    <t>test_DAQE</t>
   </si>
 </sst>
 </file>
@@ -772,7 +772,7 @@
         <v>66</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -812,7 +812,7 @@
         <v>75</v>
       </c>
       <c r="B6" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>7</v>

</xml_diff>